<commit_message>
Update echo-eg views normalization report workbook
</commit_message>
<xml_diff>
--- a/ECHO_EG_VIEWS_AND_PLAX_NORMALIZATION_REPORT.xlsx
+++ b/ECHO_EG_VIEWS_AND_PLAX_NORMALIZATION_REPORT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\houra\Desktop\echo-view-labels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1DE983-7932-4036-AC4B-1B797E5DF877}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C1D5A6D-C8FB-4E4D-A227-BC6F20F9F2EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="36">
   <si>
     <t>P10-MP4</t>
   </si>
@@ -102,6 +102,33 @@
   </si>
   <si>
     <t>Count</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>A2C +1</t>
+  </si>
+  <si>
+    <t>A3C +1</t>
+  </si>
+  <si>
+    <t>A4C +1</t>
+  </si>
+  <si>
+    <t>A5C +1</t>
+  </si>
+  <si>
+    <t>PLAX +1</t>
+  </si>
+  <si>
+    <t>PSAX_AP +1</t>
+  </si>
+  <si>
+    <t>PSAX_AV +1</t>
+  </si>
+  <si>
+    <t>PSAX_MV +1</t>
   </si>
 </sst>
 </file>
@@ -122,7 +149,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -139,6 +166,18 @@
         <fgColor rgb="FFEAF2E3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -152,7 +191,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -164,6 +203,8 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -466,7 +507,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="4" width="28" customWidth="1"/>
@@ -599,45 +640,132 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="A10" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="5" t="s">
         <v>20</v>
       </c>
+      <c r="D10" s="5" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="A11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="5" t="s">
         <v>24</v>
       </c>
+      <c r="D11" s="5" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="A12" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C13" t="s">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C14" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>